<commit_message>
Speaker diarization is LLM-only
</commit_message>
<xml_diff>
--- a/exports/sales_call_report.xlsx
+++ b/exports/sales_call_report.xlsx
@@ -185,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -202,6 +202,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -541,7 +544,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:W9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -731,6 +734,16 @@
       <c r="I7" s="5"/>
       <c r="W7" s="4"/>
     </row>
+    <row r="8" ht="18" customHeight="1" spans="7:23" x14ac:dyDescent="0.25">
+      <c r="G8" s="2"/>
+      <c r="I8" s="5"/>
+      <c r="W8" s="4"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" spans="7:23" x14ac:dyDescent="0.25">
+      <c r="G9" s="7"/>
+      <c r="I9" s="8"/>
+      <c r="W9" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>